<commit_message>
New function for package
</commit_message>
<xml_diff>
--- a/Data/Referentieprijzen hoofdstuk 4.xlsx
+++ b/Data/Referentieprijzen hoofdstuk 4.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveeur-my.sharepoint.com/personal/85304spe_eur_nl/Documents/Documents/TforT/TforT-package/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{074845F6-8515-4A77-9F76-85451BF89FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EFBBAEC-23C1-4E39-8761-6A479DE64CFF}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{074845F6-8515-4A77-9F76-85451BF89FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{868D0B4E-DB19-4844-897C-834C4F3B5F13}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2200" yWindow="2200" windowWidth="14400" windowHeight="7360" xr2:uid="{E853C0CD-6CE5-4AEA-AAF5-49787F8E4E8C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{E853C0CD-6CE5-4AEA-AAF5-49787F8E4E8C}"/>
   </bookViews>
   <sheets>
     <sheet name="tab_iMCQ" sheetId="1" r:id="rId1"/>
+    <sheet name="tab_iPCQ" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Eenheid</t>
   </si>
@@ -117,6 +118,12 @@
   </si>
   <si>
     <t>Vervangingskosten voor huishoudelijk werk</t>
+  </si>
+  <si>
+    <t>Productiviteitskosten per uur per betaald werkende</t>
+  </si>
+  <si>
+    <t>Vervangingskosten per uur</t>
   </si>
 </sst>
 </file>
@@ -237,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -255,6 +262,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -790,4 +803,43 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21F64048-DF20-4A94-9819-69C98AFEA818}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="22.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="8">
+        <v>39.880000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="8">
+        <v>18.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Inclusion of Tic-P function and adjustments in iMCQ function
</commit_message>
<xml_diff>
--- a/Data/Referentieprijzen hoofdstuk 4.xlsx
+++ b/Data/Referentieprijzen hoofdstuk 4.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveeur-my.sharepoint.com/personal/85304spe_eur_nl/Documents/Documents/TforT/TforT-package/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{074845F6-8515-4A77-9F76-85451BF89FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{868D0B4E-DB19-4844-897C-834C4F3B5F13}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{074845F6-8515-4A77-9F76-85451BF89FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2CDAAF7-C33B-45A7-95FF-CB1CFF2F6F97}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{E853C0CD-6CE5-4AEA-AAF5-49787F8E4E8C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{E853C0CD-6CE5-4AEA-AAF5-49787F8E4E8C}"/>
   </bookViews>
   <sheets>
     <sheet name="tab_iMCQ" sheetId="1" r:id="rId1"/>
     <sheet name="tab_iPCQ" sheetId="2" r:id="rId2"/>
+    <sheet name="tab_Tic-P" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="32">
   <si>
     <t>Eenheid</t>
   </si>
@@ -124,6 +125,15 @@
   </si>
   <si>
     <t>Vervangingskosten per uur</t>
+  </si>
+  <si>
+    <t>POH-GGZ, Groepsconsult</t>
+  </si>
+  <si>
+    <t>Consult zorgverlener in de PAAZ/PUK</t>
+  </si>
+  <si>
+    <t>Consult zorgverlener in de specialistische GGZ-instellingen</t>
   </si>
 </sst>
 </file>
@@ -842,4 +852,252 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5217451-19D4-4262-A2D9-5C3921C36A3C}">
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.7265625" customWidth="1"/>
+    <col min="2" max="2" width="26.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="4">
+        <v>43.31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="4">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="4">
+        <v>38.89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4">
+        <v>24.32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4">
+        <v>40.93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="54.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4">
+        <v>98.61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="63.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="4">
+        <v>43.31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4">
+        <v>32.76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4">
+        <v>57.58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4">
+        <v>30.64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="4">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="4">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="4">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4">
+        <v>83.29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="54.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="45.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22" s="4">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="54.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="72.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="4">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="4">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="6">
+        <v>18.8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="8">
+        <v>140</v>
+      </c>
+      <c r="C28" s="8"/>
+    </row>
+    <row r="29" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="8">
+        <v>134</v>
+      </c>
+      <c r="C29" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changes in ipcq function
</commit_message>
<xml_diff>
--- a/Data/Referentieprijzen hoofdstuk 4.xlsx
+++ b/Data/Referentieprijzen hoofdstuk 4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveeur-my.sharepoint.com/personal/85304spe_eur_nl/Documents/Documents/TforT/TforT-package/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{074845F6-8515-4A77-9F76-85451BF89FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0DA7B3D-B8F0-44C2-8481-611C3A574CF7}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{074845F6-8515-4A77-9F76-85451BF89FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B14E615A-C26E-4169-BF87-3DD372D31AD0}"/>
   <bookViews>
-    <workbookView xWindow="-3876" yWindow="-17388" windowWidth="30936" windowHeight="16896" activeTab="2" xr2:uid="{E853C0CD-6CE5-4AEA-AAF5-49787F8E4E8C}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7360" xr2:uid="{E853C0CD-6CE5-4AEA-AAF5-49787F8E4E8C}"/>
   </bookViews>
   <sheets>
     <sheet name="tab_iMCQ" sheetId="1" r:id="rId1"/>
@@ -263,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -288,6 +288,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -603,14 +606,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7EE5066-EA4D-4511-BCCC-C303DA2A6C71}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.54296875" customWidth="1"/>
     <col min="2" max="2" width="27.453125" customWidth="1"/>
+    <col min="7" max="7" width="58.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -618,15 +622,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="4">
-        <v>43.31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>30.87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -634,7 +638,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -642,15 +646,16 @@
         <v>38.89</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="4">
         <v>24.32</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G5" s="9"/>
+    </row>
+    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
@@ -658,7 +663,7 @@
         <v>40.93</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -666,7 +671,7 @@
         <v>24.7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -674,7 +679,7 @@
         <v>98.61</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
@@ -682,7 +687,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
@@ -690,7 +695,7 @@
         <v>43.31</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
@@ -698,7 +703,7 @@
         <v>32.76</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -706,7 +711,7 @@
         <v>57.58</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -714,7 +719,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
@@ -722,7 +727,7 @@
         <v>30.64</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>5</v>
       </c>
@@ -730,7 +735,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>6</v>
       </c>
@@ -830,7 +835,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.1796875" customWidth="1"/>
-    <col min="2" max="2" width="22.90625" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -865,14 +870,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5217451-19D4-4262-A2D9-5C3921C36A3C}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.54296875" customWidth="1"/>
     <col min="2" max="2" width="26.453125" customWidth="1"/>
+    <col min="9" max="9" width="70.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -880,7 +886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="7" t="s">
         <v>32</v>
       </c>
@@ -888,7 +894,7 @@
         <v>30.87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -896,7 +902,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -904,7 +910,7 @@
         <v>38.89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -912,15 +918,16 @@
         <v>24.32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="4">
         <v>40.93</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="I6" s="9"/>
+    </row>
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -928,7 +935,7 @@
         <v>24.7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>34</v>
       </c>
@@ -936,7 +943,7 @@
         <v>98.61</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
@@ -944,7 +951,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -952,7 +959,7 @@
         <v>98.61</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
@@ -961,7 +968,7 @@
       </c>
       <c r="C11" s="8"/>
     </row>
-    <row r="12" spans="1:3" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:9" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="7" t="s">
         <v>31</v>
       </c>
@@ -970,7 +977,7 @@
       </c>
       <c r="C12" s="8"/>
     </row>
-    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="7" t="s">
         <v>29</v>
       </c>
@@ -978,7 +985,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="7" t="s">
         <v>33</v>
       </c>
@@ -986,7 +993,7 @@
         <v>30.87</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
@@ -994,7 +1001,7 @@
         <v>32.76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>

</xml_diff>